<commit_message>
code done for the cloud data warehouse connection in 5-12-25
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -3,7 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C4075D25-79A4-4412-8C25-65253FCA65CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8952F47E-C00F-4E4A-AFB0-739B6657AD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,7 +17,6 @@
     <sheet name="Import Template" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:P18"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -22,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="29">
   <si>
     <t>ruleType</t>
   </si>
@@ -94,6 +98,21 @@
   </si>
   <si>
     <t>Data Pushdown Validation - Import SQL</t>
+  </si>
+  <si>
+    <t>connectionType</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>Cloud Data Warehouse</t>
+  </si>
+  <si>
+    <t>regression_database</t>
+  </si>
+  <si>
+    <t>Redshift-with-jdbc-UserConn</t>
   </si>
 </sst>
 </file>
@@ -137,13 +156,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -425,19 +447,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="56" customWidth="1"/>
     <col min="3" max="3" width="22.42578125" customWidth="1"/>
     <col min="4" max="4" width="24.140625" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="6" max="6" width="29.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.85546875" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,16 +474,19 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -474,16 +500,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -497,16 +526,19 @@
         <v>10</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -520,16 +552,19 @@
         <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -543,12 +578,119 @@
         <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -559,17 +701,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF74396-CAE9-4386-83E8-43C18AE860D9}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" customWidth="1"/>
     <col min="2" max="2" width="62.42578125" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="4" max="4" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="27.5703125" customWidth="1"/>
+    <col min="6" max="6" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -583,10 +726,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -600,10 +746,13 @@
         <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -617,10 +766,13 @@
         <v>10</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -634,10 +786,13 @@
         <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -651,7 +806,90 @@
         <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Code change at office 11-12-25
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B6A40A1-659E-4C0E-B459-AB4BD24E7E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B911321C-808C-436A-ADC1-FE49BF3FD97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Mapping test case ID with each execution
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B5914A-0895-4156-8CEB-99F4273D4A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCBE6FA-135C-412D-8866-179891E98E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="45">
   <si>
     <t>ruleType</t>
   </si>
@@ -135,6 +135,33 @@
   </si>
   <si>
     <t>AD-Workflow</t>
+  </si>
+  <si>
+    <t>xrayTestId</t>
+  </si>
+  <si>
+    <t>NRR-41671</t>
+  </si>
+  <si>
+    <t>NRR-41672</t>
+  </si>
+  <si>
+    <t>NRR-41673</t>
+  </si>
+  <si>
+    <t>NRR-41674</t>
+  </si>
+  <si>
+    <t>NRR-41675</t>
+  </si>
+  <si>
+    <t>NRR-41676</t>
+  </si>
+  <si>
+    <t>NRR-41677</t>
+  </si>
+  <si>
+    <t>NRR-41678</t>
   </si>
 </sst>
 </file>
@@ -478,7 +505,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
@@ -490,9 +517,10 @@
     <col min="7" max="7" width="34.42578125" customWidth="1"/>
     <col min="8" max="8" width="21" customWidth="1"/>
     <col min="9" max="9" width="12.140625" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -520,8 +548,11 @@
       <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -549,8 +580,11 @@
       <c r="I2" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -578,8 +612,11 @@
       <c r="I3" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -607,8 +644,11 @@
       <c r="I4" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
@@ -636,8 +676,11 @@
       <c r="I5" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -665,8 +708,11 @@
       <c r="I6" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -694,8 +740,11 @@
       <c r="I7" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
@@ -723,8 +772,11 @@
       <c r="I8" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
@@ -751,6 +803,9 @@
       </c>
       <c r="I9" s="2" t="s">
         <v>10</v>
+      </c>
+      <c r="J9" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
done all changes in the template level
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCBE6FA-135C-412D-8866-179891E98E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4A51EA-128C-4E75-8BB6-B50CE3FDA097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -56,9 +56,6 @@
     <t>Test_Generator-WIP</t>
   </si>
   <si>
-    <t>public</t>
-  </si>
-  <si>
     <t>staff</t>
   </si>
   <si>
@@ -107,21 +104,12 @@
     <t>File</t>
   </si>
   <si>
-    <t>AD-Test</t>
-  </si>
-  <si>
     <t>SourceConnectionName</t>
   </si>
   <si>
     <t>TargetConnectionName</t>
   </si>
   <si>
-    <t>Postgresql-without-jdbc-SysConn</t>
-  </si>
-  <si>
-    <t>Postgresql-without-jdbc-UserConn</t>
-  </si>
-  <si>
     <t>Redshift-without-jdbc-SysConn</t>
   </si>
   <si>
@@ -162,6 +150,18 @@
   </si>
   <si>
     <t>NRR-41678</t>
+  </si>
+  <si>
+    <t>7-4-0</t>
+  </si>
+  <si>
+    <t>Mysql-with-jdbc-SysConn</t>
+  </si>
+  <si>
+    <t>Mysql-with-jdbc-UserConn</t>
+  </si>
+  <si>
+    <t>icedq</t>
   </si>
 </sst>
 </file>
@@ -534,13 +534,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
@@ -549,7 +549,7 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -563,121 +563,121 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="J2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="J3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="J4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="J5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -691,121 +691,121 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="C7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="I7" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="C8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="I8" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="C9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="I9" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -843,13 +843,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -857,91 +857,91 @@
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -949,91 +949,91 @@
         <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1041,91 +1041,91 @@
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1162,13 +1162,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
@@ -1188,22 +1188,22 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added rule in existing workflow
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4A51EA-128C-4E75-8BB6-B50CE3FDA097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774DB471-4375-4845-8247-04328B4FFBA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
     <sheet name="Import Template" sheetId="2" r:id="rId2"/>
     <sheet name="Workflow" sheetId="3" r:id="rId3"/>
+    <sheet name="Exsiting Workflow" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="47">
   <si>
     <t>ruleType</t>
   </si>
@@ -162,6 +163,12 @@
   </si>
   <si>
     <t>icedq</t>
+  </si>
+  <si>
+    <t>workflowName</t>
+  </si>
+  <si>
+    <t>Workflow - All rules type</t>
   </si>
 </sst>
 </file>
@@ -1135,7 +1142,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F87908C9-FFD2-452C-9D55-9D6FE8A0B684}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1146,9 +1153,10 @@
     <col min="6" max="7" width="32.7109375" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="11" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1176,8 +1184,11 @@
       <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1204,6 +1215,95 @@
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{632888C4-28F7-4A93-B393-A9F2EBCE0EDF}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a excel connection support
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774DB471-4375-4845-8247-04328B4FFBA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDB6BA3-5E2D-4909-89F3-CA2702B3E661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
     <sheet name="Import Template" sheetId="2" r:id="rId2"/>
-    <sheet name="Workflow" sheetId="3" r:id="rId3"/>
+    <sheet name="Create Workflow" sheetId="3" r:id="rId3"/>
     <sheet name="Exsiting Workflow" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="49">
   <si>
     <t>ruleType</t>
   </si>
@@ -117,65 +117,71 @@
     <t>Redshift-without-jdbc-UserConn</t>
   </si>
   <si>
+    <t>AD-Workflow</t>
+  </si>
+  <si>
+    <t>xrayTestId</t>
+  </si>
+  <si>
+    <t>NRR-41671</t>
+  </si>
+  <si>
+    <t>NRR-41672</t>
+  </si>
+  <si>
+    <t>NRR-41673</t>
+  </si>
+  <si>
+    <t>NRR-41674</t>
+  </si>
+  <si>
+    <t>NRR-41675</t>
+  </si>
+  <si>
+    <t>NRR-41676</t>
+  </si>
+  <si>
+    <t>NRR-41677</t>
+  </si>
+  <si>
+    <t>NRR-41678</t>
+  </si>
+  <si>
+    <t>Mysql-with-jdbc-SysConn</t>
+  </si>
+  <si>
+    <t>Mysql-with-jdbc-UserConn</t>
+  </si>
+  <si>
+    <t>icedq</t>
+  </si>
+  <si>
+    <t>workflowName</t>
+  </si>
+  <si>
+    <t>Workflow - All rules type</t>
+  </si>
+  <si>
+    <t>7-5-0</t>
+  </si>
+  <si>
+    <t>Excel_Azure_Location_Azure_Access_Key--SysConn</t>
+  </si>
+  <si>
+    <t>Excel_Azure_Location_Azure_Access_Key--UserConn</t>
+  </si>
+  <si>
     <t>FlatFileSQL-S3-AWS-IAM-SysConn</t>
   </si>
   <si>
     <t>FlatFileSQL-S3-AWS-IAM-UserConn</t>
-  </si>
-  <si>
-    <t>AD-Workflow</t>
-  </si>
-  <si>
-    <t>xrayTestId</t>
-  </si>
-  <si>
-    <t>NRR-41671</t>
-  </si>
-  <si>
-    <t>NRR-41672</t>
-  </si>
-  <si>
-    <t>NRR-41673</t>
-  </si>
-  <si>
-    <t>NRR-41674</t>
-  </si>
-  <si>
-    <t>NRR-41675</t>
-  </si>
-  <si>
-    <t>NRR-41676</t>
-  </si>
-  <si>
-    <t>NRR-41677</t>
-  </si>
-  <si>
-    <t>NRR-41678</t>
-  </si>
-  <si>
-    <t>7-4-0</t>
-  </si>
-  <si>
-    <t>Mysql-with-jdbc-SysConn</t>
-  </si>
-  <si>
-    <t>Mysql-with-jdbc-UserConn</t>
-  </si>
-  <si>
-    <t>icedq</t>
-  </si>
-  <si>
-    <t>workflowName</t>
-  </si>
-  <si>
-    <t>Workflow - All rules type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +199,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -218,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -231,6 +244,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -556,7 +572,7 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -570,25 +586,25 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -602,25 +618,25 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -634,25 +650,25 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -666,25 +682,25 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -698,7 +714,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -716,7 +732,7 @@
         <v>9</v>
       </c>
       <c r="J6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -730,7 +746,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -748,7 +764,7 @@
         <v>9</v>
       </c>
       <c r="J7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -762,7 +778,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -780,7 +796,7 @@
         <v>9</v>
       </c>
       <c r="J8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -794,7 +810,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -812,7 +828,7 @@
         <v>9</v>
       </c>
       <c r="J9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -824,7 +840,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF74396-CAE9-4386-83E8-43C18AE860D9}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
@@ -832,7 +848,7 @@
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="4" max="4" width="15.140625" customWidth="1"/>
     <col min="5" max="5" width="23.140625" customWidth="1"/>
-    <col min="6" max="6" width="32.140625" customWidth="1"/>
+    <col min="6" max="6" width="46.85546875" customWidth="1"/>
     <col min="7" max="7" width="32.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -870,16 +886,16 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -893,16 +909,16 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -916,16 +932,16 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -939,16 +955,16 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -962,7 +978,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -985,7 +1001,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -1008,7 +1024,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -1031,7 +1047,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -1043,96 +1059,188 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="F10" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>30</v>
+      <c r="F11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>29</v>
+      <c r="F12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E13" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>29</v>
+      <c r="F13" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1185,7 +1293,7 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -1199,25 +1307,25 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1271,7 +1379,7 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1285,25 +1393,25 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add exccel file logic
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDB6BA3-5E2D-4909-89F3-CA2702B3E661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6722B347-FF08-4F81-9C78-92BF8B4899F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="52">
   <si>
     <t>ruleType</t>
   </si>
@@ -162,9 +162,6 @@
     <t>Workflow - All rules type</t>
   </si>
   <si>
-    <t>7-5-0</t>
-  </si>
-  <si>
     <t>Excel_Azure_Location_Azure_Access_Key--SysConn</t>
   </si>
   <si>
@@ -175,6 +172,18 @@
   </si>
   <si>
     <t>FlatFileSQL-S3-AWS-IAM-UserConn</t>
+  </si>
+  <si>
+    <t>fileType</t>
+  </si>
+  <si>
+    <t>FlatFile-SQL</t>
+  </si>
+  <si>
+    <t>Excel</t>
+  </si>
+  <si>
+    <t>AD-Test</t>
   </si>
 </sst>
 </file>
@@ -586,7 +595,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -618,7 +627,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -650,7 +659,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -682,7 +691,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -714,7 +723,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -746,7 +755,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -778,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -810,7 +819,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -840,19 +849,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF74396-CAE9-4386-83E8-43C18AE860D9}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
     <col min="2" max="2" width="55.140625" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.140625" customWidth="1"/>
-    <col min="6" max="6" width="46.85546875" customWidth="1"/>
-    <col min="7" max="7" width="32.28515625" customWidth="1"/>
+    <col min="5" max="6" width="23.140625" customWidth="1"/>
+    <col min="7" max="7" width="46.85546875" customWidth="1"/>
+    <col min="8" max="8" width="32.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -869,13 +878,16 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -886,19 +898,20 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="2"/>
+      <c r="G2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -909,19 +922,20 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -932,19 +946,20 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -955,19 +970,20 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -978,19 +994,20 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2"/>
+      <c r="G6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -1001,19 +1018,20 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2"/>
+      <c r="G7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
@@ -1024,19 +1042,20 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="F8" s="2"/>
       <c r="G8" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -1047,19 +1066,20 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="F9" s="2"/>
       <c r="G9" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
@@ -1070,19 +1090,22 @@
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
@@ -1093,19 +1116,22 @@
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -1116,19 +1142,22 @@
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>14</v>
       </c>
@@ -1139,19 +1168,22 @@
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>6</v>
       </c>
@@ -1162,19 +1194,22 @@
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>10</v>
       </c>
@@ -1185,19 +1220,22 @@
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G15" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -1208,19 +1246,22 @@
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H16" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -1231,19 +1272,23 @@
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>45</v>
+      <c r="H17" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1296,7 +1341,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
26-2-26 changes At Office
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6722B347-FF08-4F81-9C78-92BF8B4899F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF03DAEB-67EF-40ED-AC85-2073A701FC1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -168,12 +168,6 @@
     <t>Excel_Azure_Location_Azure_Access_Key--UserConn</t>
   </si>
   <si>
-    <t>FlatFileSQL-S3-AWS-IAM-SysConn</t>
-  </si>
-  <si>
-    <t>FlatFileSQL-S3-AWS-IAM-UserConn</t>
-  </si>
-  <si>
     <t>fileType</t>
   </si>
   <si>
@@ -184,6 +178,12 @@
   </si>
   <si>
     <t>AD-Test</t>
+  </si>
+  <si>
+    <t>FlatFile-SQL_S3_Location_AWS-IAM--SysConn</t>
+  </si>
+  <si>
+    <t>FlatFile-SQL_S3_Location_AWS-IAM--UserConn</t>
   </si>
 </sst>
 </file>
@@ -595,7 +595,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -627,7 +627,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -659,7 +659,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -691,7 +691,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -723,7 +723,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -755,7 +755,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -819,7 +819,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -857,8 +857,8 @@
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="4" max="4" width="15.140625" customWidth="1"/>
     <col min="5" max="6" width="23.140625" customWidth="1"/>
-    <col min="7" max="7" width="46.85546875" customWidth="1"/>
-    <col min="8" max="8" width="32.28515625" customWidth="1"/>
+    <col min="7" max="7" width="46.28515625" customWidth="1"/>
+    <col min="8" max="8" width="47.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -878,7 +878,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>25</v>
@@ -887,7 +887,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -898,7 +898,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -911,7 +911,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -922,7 +922,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -946,7 +946,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -970,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -994,7 +994,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -1018,7 +1018,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -1042,7 +1042,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -1066,7 +1066,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -1079,7 +1079,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
@@ -1090,22 +1090,22 @@
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
@@ -1116,19 +1116,19 @@
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1142,19 +1142,19 @@
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1168,19 +1168,19 @@
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1194,13 +1194,13 @@
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>44</v>
@@ -1220,13 +1220,13 @@
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>44</v>
@@ -1246,13 +1246,13 @@
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>44</v>
@@ -1272,13 +1272,13 @@
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
Jenkins parameter changes are done
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF03DAEB-67EF-40ED-AC85-2073A701FC1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD1E552-E0BB-4871-8A95-7D0FF25023E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -177,13 +177,13 @@
     <t>Excel</t>
   </si>
   <si>
-    <t>AD-Test</t>
-  </si>
-  <si>
     <t>FlatFile-SQL_S3_Location_AWS-IAM--SysConn</t>
   </si>
   <si>
     <t>FlatFile-SQL_S3_Location_AWS-IAM--UserConn</t>
+  </si>
+  <si>
+    <t>7-4-4</t>
   </si>
 </sst>
 </file>
@@ -595,7 +595,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -627,7 +627,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -659,7 +659,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -691,7 +691,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -723,7 +723,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -755,7 +755,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -819,7 +819,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -898,7 +898,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -922,7 +922,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -946,7 +946,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -970,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -994,7 +994,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -1018,7 +1018,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -1042,7 +1042,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -1066,7 +1066,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -1090,7 +1090,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>24</v>
@@ -1099,10 +1099,10 @@
         <v>47</v>
       </c>
       <c r="G10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1116,7 +1116,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
@@ -1125,10 +1125,10 @@
         <v>47</v>
       </c>
       <c r="G11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1142,7 +1142,7 @@
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>24</v>
@@ -1151,10 +1151,10 @@
         <v>47</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1168,7 +1168,7 @@
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>24</v>
@@ -1177,10 +1177,10 @@
         <v>47</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1194,7 +1194,7 @@
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>24</v>
@@ -1220,7 +1220,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>24</v>
@@ -1246,7 +1246,7 @@
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>24</v>
@@ -1272,7 +1272,7 @@
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>24</v>
@@ -1395,7 +1395,7 @@
     <col min="10" max="10" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
made a changes in the sendmail file
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\ICEDQ-TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E448DB-7E9B-4E64-B33C-3A99A86EC0CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4255D5-BE17-4165-9BD3-79E385E3C51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
     <t>FlatFile-SQL_S3_Location_AWS-IAM--UserConn</t>
   </si>
   <si>
-    <t>7-4-4</t>
+    <t>7-5-3</t>
   </si>
 </sst>
 </file>
@@ -538,21 +538,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" customWidth="1"/>
-    <col min="2" max="2" width="53.85546875" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" customWidth="1"/>
-    <col min="6" max="6" width="32.7109375" customWidth="1"/>
-    <col min="7" max="7" width="34.42578125" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="53.88671875" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="7" max="7" width="34.44140625" customWidth="1"/>
     <col min="8" max="8" width="21" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.109375" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -584,7 +584,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -616,7 +616,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -648,7 +648,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -680,7 +680,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -712,7 +712,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -744,7 +744,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -776,7 +776,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
@@ -808,7 +808,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -850,18 +850,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF74396-CAE9-4386-83E8-43C18AE860D9}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="55.140625" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="6" width="23.140625" customWidth="1"/>
-    <col min="7" max="7" width="46.28515625" customWidth="1"/>
-    <col min="8" max="8" width="47.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="55.109375" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" customWidth="1"/>
+    <col min="5" max="6" width="23.109375" customWidth="1"/>
+    <col min="7" max="7" width="46.33203125" customWidth="1"/>
+    <col min="8" max="8" width="47.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -887,7 +887,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -911,7 +911,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -935,7 +935,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -959,7 +959,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -983,7 +983,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
@@ -1105,7 +1105,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>14</v>
       </c>
@@ -1183,7 +1183,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>6</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>10</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -1296,20 +1296,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F87908C9-FFD2-452C-9D55-9D6FE8A0B684}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="36.85546875" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="6" max="7" width="32.7109375" customWidth="1"/>
+    <col min="2" max="2" width="36.88671875" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="7" width="32.6640625" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="11" width="25.5703125" customWidth="1"/>
+    <col min="10" max="11" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1381,21 +1381,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{632888C4-28F7-4A93-B393-A9F2EBCE0EDF}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.44140625" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
just small changes not a improvment
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\ICEDQ-TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4255D5-BE17-4165-9BD3-79E385E3C51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B91BAD-329C-4901-A446-866AED11A14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="53">
   <si>
     <t>ruleType</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>7-5-3</t>
+  </si>
+  <si>
+    <t>7-6.0</t>
   </si>
 </sst>
 </file>
@@ -898,7 +901,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -922,7 +925,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -946,7 +949,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -970,7 +973,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -994,7 +997,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -1018,7 +1021,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -1042,7 +1045,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -1066,7 +1069,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -1090,7 +1093,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>24</v>
@@ -1116,7 +1119,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
@@ -1142,7 +1145,7 @@
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>24</v>
@@ -1168,7 +1171,7 @@
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>24</v>
@@ -1194,7 +1197,7 @@
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>24</v>
@@ -1220,7 +1223,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>24</v>
@@ -1246,7 +1249,7 @@
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>24</v>
@@ -1272,7 +1275,7 @@
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
Added new changes according to new release
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\ICEDQ-TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B91BAD-329C-4901-A446-866AED11A14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46A0F5A6-2D0C-4C57-A962-BD98CC985786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="54">
   <si>
     <t>ruleType</t>
   </si>
@@ -186,7 +186,10 @@
     <t>7-5-3</t>
   </si>
   <si>
-    <t>7-6.0</t>
+    <t>accountName</t>
+  </si>
+  <si>
+    <t>Quality_Assurance</t>
   </si>
 </sst>
 </file>
@@ -540,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -553,9 +556,10 @@
     <col min="8" max="8" width="21" customWidth="1"/>
     <col min="9" max="9" width="12.109375" customWidth="1"/>
     <col min="10" max="10" width="14.88671875" customWidth="1"/>
+    <col min="11" max="11" width="18.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -586,8 +590,11 @@
       <c r="J1" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -607,7 +614,7 @@
         <v>39</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>41</v>
@@ -618,8 +625,11 @@
       <c r="J2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -639,7 +649,7 @@
         <v>39</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>41</v>
@@ -650,8 +660,11 @@
       <c r="J3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -682,8 +695,11 @@
       <c r="J4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -714,8 +730,11 @@
       <c r="J5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -735,7 +754,7 @@
         <v>27</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>23</v>
@@ -746,8 +765,11 @@
       <c r="J6" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -767,7 +789,7 @@
         <v>27</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>23</v>
@@ -778,8 +800,11 @@
       <c r="J7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
@@ -810,8 +835,11 @@
       <c r="J8" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -841,6 +869,9 @@
       </c>
       <c r="J9" t="s">
         <v>38</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -852,7 +883,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF74396-CAE9-4386-83E8-43C18AE860D9}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
@@ -862,9 +893,10 @@
     <col min="5" max="6" width="23.109375" customWidth="1"/>
     <col min="7" max="7" width="46.33203125" customWidth="1"/>
     <col min="8" max="8" width="47.88671875" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -889,8 +921,11 @@
       <c r="H1" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -901,7 +936,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -913,8 +948,11 @@
       <c r="H2" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I2" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -925,7 +963,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -937,8 +975,11 @@
       <c r="H3" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I3" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -949,7 +990,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -961,8 +1002,11 @@
       <c r="H4" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I4" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -973,7 +1017,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -985,8 +1029,11 @@
       <c r="H5" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I5" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -997,7 +1044,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -1009,8 +1056,11 @@
       <c r="H6" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I6" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -1021,7 +1071,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -1033,8 +1083,11 @@
       <c r="H7" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I7" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
@@ -1045,7 +1098,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -1057,8 +1110,11 @@
       <c r="H8" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I8" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -1069,7 +1125,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -1081,8 +1137,11 @@
       <c r="H9" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I9" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
@@ -1093,7 +1152,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>24</v>
@@ -1107,8 +1166,11 @@
       <c r="H10" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I10" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
@@ -1119,7 +1181,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
@@ -1133,8 +1195,11 @@
       <c r="H11" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I11" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -1145,7 +1210,7 @@
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>24</v>
@@ -1159,8 +1224,11 @@
       <c r="H12" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I12" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>14</v>
       </c>
@@ -1171,7 +1239,7 @@
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>24</v>
@@ -1185,8 +1253,11 @@
       <c r="H13" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I13" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>6</v>
       </c>
@@ -1197,7 +1268,7 @@
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>24</v>
@@ -1211,8 +1282,11 @@
       <c r="H14" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I14" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>10</v>
       </c>
@@ -1223,7 +1297,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>24</v>
@@ -1237,8 +1311,11 @@
       <c r="H15" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I15" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -1249,7 +1326,7 @@
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>24</v>
@@ -1263,8 +1340,11 @@
       <c r="H16" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I16" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -1275,7 +1355,7 @@
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>24</v>
@@ -1288,6 +1368,9 @@
       </c>
       <c r="H17" s="2" t="s">
         <v>44</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1298,7 +1381,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F87908C9-FFD2-452C-9D55-9D6FE8A0B684}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1312,7 +1395,7 @@
     <col min="10" max="11" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1343,8 +1426,11 @@
       <c r="J1" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1364,7 +1450,7 @@
         <v>39</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>41</v>
@@ -1374,6 +1460,9 @@
       </c>
       <c r="J2" s="2" t="s">
         <v>43</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1383,7 +1472,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{632888C4-28F7-4A93-B393-A9F2EBCE0EDF}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -1396,9 +1485,10 @@
     <col min="8" max="8" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="26.5546875" customWidth="1"/>
+    <col min="11" max="11" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1429,8 +1519,11 @@
       <c r="J1" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1450,7 +1543,7 @@
         <v>39</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>41</v>
@@ -1460,6 +1553,9 @@
       </c>
       <c r="J2" s="2" t="s">
         <v>43</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add changes for new release 7.6.0
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\ICEDQ-TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46A0F5A6-2D0C-4C57-A962-BD98CC985786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E77BE29-87D8-4356-BED3-A37F4C3E07F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="50">
   <si>
     <t>ruleType</t>
   </si>
@@ -114,9 +114,6 @@
     <t>Redshift-without-jdbc-SysConn</t>
   </si>
   <si>
-    <t>Redshift-without-jdbc-UserConn</t>
-  </si>
-  <si>
     <t>AD-Workflow</t>
   </si>
   <si>
@@ -150,9 +147,6 @@
     <t>Mysql-with-jdbc-SysConn</t>
   </si>
   <si>
-    <t>Mysql-with-jdbc-UserConn</t>
-  </si>
-  <si>
     <t>icedq</t>
   </si>
   <si>
@@ -165,9 +159,6 @@
     <t>Excel_Azure_Location_Azure_Access_Key--SysConn</t>
   </si>
   <si>
-    <t>Excel_Azure_Location_Azure_Access_Key--UserConn</t>
-  </si>
-  <si>
     <t>fileType</t>
   </si>
   <si>
@@ -180,16 +171,13 @@
     <t>FlatFile-SQL_S3_Location_AWS-IAM--SysConn</t>
   </si>
   <si>
-    <t>FlatFile-SQL_S3_Location_AWS-IAM--UserConn</t>
-  </si>
-  <si>
     <t>7-5-3</t>
   </si>
   <si>
     <t>accountName</t>
   </si>
   <si>
-    <t>Quality_Assurance</t>
+    <t>TestGenerator</t>
   </si>
 </sst>
 </file>
@@ -588,10 +576,10 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -605,28 +593,28 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -640,28 +628,28 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -675,28 +663,28 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -710,28 +698,28 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -745,7 +733,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -763,10 +751,10 @@
         <v>9</v>
       </c>
       <c r="J6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -780,7 +768,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -798,10 +786,10 @@
         <v>9</v>
       </c>
       <c r="J7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -815,7 +803,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -833,10 +821,10 @@
         <v>9</v>
       </c>
       <c r="J8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -850,7 +838,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -868,10 +856,10 @@
         <v>9</v>
       </c>
       <c r="J9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -913,7 +901,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>25</v>
@@ -922,7 +910,7 @@
         <v>26</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -936,20 +924,20 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -963,20 +951,20 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -990,20 +978,20 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1017,20 +1005,20 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -1044,7 +1032,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -1054,10 +1042,10 @@
         <v>27</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1071,7 +1059,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -1081,10 +1069,10 @@
         <v>27</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -1098,7 +1086,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -1111,7 +1099,7 @@
         <v>27</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -1125,7 +1113,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -1138,7 +1126,7 @@
         <v>27</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1152,22 +1140,22 @@
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -1181,22 +1169,22 @@
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -1210,22 +1198,22 @@
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -1239,22 +1227,22 @@
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -1268,22 +1256,22 @@
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -1297,22 +1285,22 @@
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -1326,22 +1314,22 @@
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
@@ -1355,22 +1343,22 @@
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1392,7 +1380,8 @@
     <col min="6" max="7" width="32.6640625" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="11" width="25.5546875" customWidth="1"/>
+    <col min="10" max="10" width="25.5546875" customWidth="1"/>
+    <col min="11" max="11" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -1424,10 +1413,10 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1441,28 +1430,28 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1517,10 +1506,10 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1534,28 +1523,28 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
release 7.8.0 changes has been done
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\ICEDQ-TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E77BE29-87D8-4356-BED3-A37F4C3E07F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C73B33-1C25-4590-BC6C-455446841E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="58">
   <si>
     <t>ruleType</t>
   </si>
@@ -114,9 +114,6 @@
     <t>Redshift-without-jdbc-SysConn</t>
   </si>
   <si>
-    <t>AD-Workflow</t>
-  </si>
-  <si>
     <t>xrayTestId</t>
   </si>
   <si>
@@ -171,13 +168,40 @@
     <t>FlatFile-SQL_S3_Location_AWS-IAM--SysConn</t>
   </si>
   <si>
-    <t>7-5-3</t>
-  </si>
-  <si>
     <t>accountName</t>
   </si>
   <si>
-    <t>TestGenerator</t>
+    <t>duplicate</t>
+  </si>
+  <si>
+    <t>Data Duplicate Validation - Import SQL</t>
+  </si>
+  <si>
+    <t>databaseName</t>
+  </si>
+  <si>
+    <t>icedqrs</t>
+  </si>
+  <si>
+    <t>Mysql-with-jdbc-UserConn</t>
+  </si>
+  <si>
+    <t>Redshift-without-jdbc-UserConn</t>
+  </si>
+  <si>
+    <t>7-8-0</t>
+  </si>
+  <si>
+    <t>7-8-0_Workflow</t>
+  </si>
+  <si>
+    <t>Quality_Assurance</t>
+  </si>
+  <si>
+    <t>FlatFile-SQL_S3_Location_AWS-IAM--UserConn</t>
+  </si>
+  <si>
+    <t>FlatFile-SQL_Azure_Location_Azure_Access_Key--UserConn</t>
   </si>
 </sst>
 </file>
@@ -531,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -545,9 +569,10 @@
     <col min="9" max="9" width="12.109375" customWidth="1"/>
     <col min="10" max="10" width="14.88671875" customWidth="1"/>
     <col min="11" max="11" width="18.5546875" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -576,13 +601,16 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -593,31 +621,34 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -628,31 +659,34 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -663,31 +697,34 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -698,31 +735,34 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -733,7 +773,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -741,8 +781,8 @@
       <c r="F6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>27</v>
+      <c r="G6" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>23</v>
@@ -751,13 +791,16 @@
         <v>9</v>
       </c>
       <c r="J6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -768,7 +811,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -776,8 +819,8 @@
       <c r="F7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>27</v>
+      <c r="G7" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>23</v>
@@ -786,13 +829,16 @@
         <v>9</v>
       </c>
       <c r="J7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
@@ -803,7 +849,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -821,13 +867,16 @@
         <v>9</v>
       </c>
       <c r="J8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="L8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -838,7 +887,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -856,10 +905,13 @@
         <v>9</v>
       </c>
       <c r="J9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
+      </c>
+      <c r="L9" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -871,7 +923,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF74396-CAE9-4386-83E8-43C18AE860D9}">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
@@ -880,11 +932,11 @@
     <col min="4" max="4" width="15.109375" customWidth="1"/>
     <col min="5" max="6" width="23.109375" customWidth="1"/>
     <col min="7" max="7" width="46.33203125" customWidth="1"/>
-    <col min="8" max="8" width="47.88671875" customWidth="1"/>
+    <col min="8" max="8" width="56.44140625" customWidth="1"/>
     <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -901,7 +953,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>25</v>
@@ -910,7 +962,7 @@
         <v>26</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -924,20 +976,20 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -951,20 +1003,20 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -978,20 +1030,20 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1005,61 +1057,61 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="G6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>27</v>
+      <c r="G6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -1068,25 +1120,25 @@
       <c r="G7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="3" t="s">
-        <v>27</v>
+      <c r="H7" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -1095,25 +1147,25 @@
       <c r="G8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>27</v>
+      <c r="H8" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -1126,239 +1178,266 @@
         <v>27</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="A10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>46</v>
+        <v>53</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="2"/>
+      <c r="G10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>27</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="A14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>42</v>
+      <c r="H14" s="5" t="s">
+        <v>45</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1369,22 +1448,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F87908C9-FFD2-452C-9D55-9D6FE8A0B684}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="36.88671875" customWidth="1"/>
     <col min="3" max="3" width="20.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" customWidth="1"/>
     <col min="5" max="5" width="17.109375" customWidth="1"/>
     <col min="6" max="7" width="32.6640625" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="25.5546875" customWidth="1"/>
     <col min="11" max="11" width="21.6640625" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1413,13 +1493,16 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1430,28 +1513,31 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
+      </c>
+      <c r="L2" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1461,23 +1547,24 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{632888C4-28F7-4A93-B393-A9F2EBCE0EDF}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.44140625" customWidth="1"/>
     <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" customWidth="1"/>
     <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5546875" customWidth="1"/>
-    <col min="11" max="11" width="19.6640625" customWidth="1"/>
+    <col min="10" max="10" width="19.5546875" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1506,13 +1593,16 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1523,28 +1613,31 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
+      </c>
+      <c r="L2" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>